<commit_message>
Кузатув ustuni (Min_Zaxira K): X belgilangan tovar butun tizimdan chiqariladi — Power BI, buyurtma, kamomat, qidiruv, Меъёр йўқ hech qayerda chiqmaydi (Huzayfa: 'kuzatuvdan mutloq chiqarish kerak bo'lgan tovarlar bor')
</commit_message>
<xml_diff>
--- a/Minimal_zaxiralar/Min_Zaxira.xlsx
+++ b/Minimal_zaxiralar/Min_Zaxira.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -69,8 +69,12 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +109,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF8D7DA"/>
         <bgColor rgb="FFDDDDDD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -142,7 +151,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -195,6 +204,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I1408"/>
+  <dimension ref="A1:K1408"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="9" min="1" max="1"/>
@@ -524,6 +534,7 @@
     <col width="14" customWidth="1" style="9" min="6" max="6"/>
     <col width="12" customWidth="1" style="9" min="7" max="8"/>
     <col width="16" customWidth="1" style="9" min="9" max="9"/>
+    <col width="10" customWidth="1" style="10" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
@@ -570,6 +581,11 @@
       <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Ойлик_дона (тахлил)</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="inlineStr">
+        <is>
+          <t>Кузатув</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Qidiruv: min-zaxirani yashirish + meyor-yo'q tovarni aksiya deb ko'rsatish
</commit_message>
<xml_diff>
--- a/Minimal_zaxiralar/Min_Zaxira.xlsx
+++ b/Minimal_zaxiralar/Min_Zaxira.xlsx
@@ -564,37 +564,37 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="13">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Товар</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Кунлик_Истеъмол</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>Асосий_Захира</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>Цех_Захира</t>
         </is>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="D84" s="20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E84" s="18">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="D92" s="20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E92" s="18">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="D101" s="20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E101" s="18">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D103" s="20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E103" s="18">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="D145" s="20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E145" s="18">
@@ -7869,7 +7869,7 @@
       </c>
       <c r="D262" s="21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E262" s="18">
@@ -10559,7 +10559,7 @@
       </c>
       <c r="D358" s="21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E358" s="18">
@@ -18457,7 +18457,7 @@
       </c>
       <c r="D640" s="21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E640" s="18">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="D685" s="21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E685" s="18">

</xml_diff>

<commit_message>
Buyurtma: qalin List (>=1,5) yaxlitlanmaydi, List-0,4 minusovka istisno
</commit_message>
<xml_diff>
--- a/Minimal_zaxiralar/Min_Zaxira.xlsx
+++ b/Minimal_zaxiralar/Min_Zaxira.xlsx
@@ -8597,12 +8597,12 @@
       <c r="D169" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E169" s="5" t="n">
+      <c r="E169" s="5" t="str">
         <f aca="false">IF((F169+G169)&gt;0,ROUND((F169+G169)/30,2),"")</f>
-        <v>50</v>
+        <v/>
       </c>
       <c r="F169" s="5" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="G169" s="5"/>
     </row>
@@ -8665,10 +8665,10 @@
       </c>
       <c r="E172" s="5" t="n">
         <f aca="false">IF((F172+G172)&gt;0,ROUND((F172+G172)/30,2),"")</f>
-        <v>66.67</v>
+        <v>100</v>
       </c>
       <c r="F172" s="5" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G172" s="5"/>
     </row>
@@ -23070,10 +23070,10 @@
       </c>
       <c r="E827" s="5" t="n">
         <f aca="false">IF((F827+G827)&gt;0,ROUND((F827+G827)/30,2),"")</f>
-        <v>83.33</v>
+        <v>66.67</v>
       </c>
       <c r="F827" s="5" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="G827" s="5"/>
     </row>
@@ -23334,10 +23334,10 @@
       </c>
       <c r="E839" s="5" t="n">
         <f aca="false">IF((F839+G839)&gt;0,ROUND((F839+G839)/30,2),"")</f>
-        <v>16.67</v>
+        <v>20</v>
       </c>
       <c r="F839" s="5" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="G839" s="5"/>
     </row>
@@ -23508,12 +23508,12 @@
       <c r="D847" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E847" s="5" t="n">
+      <c r="E847" s="5" t="str">
         <f aca="false">IF((F847+G847)&gt;0,ROUND((F847+G847)/30,2),"")</f>
-        <v>5</v>
+        <v/>
       </c>
       <c r="F847" s="5" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="G847" s="5"/>
     </row>

</xml_diff>

<commit_message>
Buyurtma: yirik tovarlar (List>=1,5, Truba>76, Profil 60+) yaxlitlanmaydi, List-0,4 minusovka istisno
</commit_message>
<xml_diff>
--- a/Minimal_zaxiralar/Min_Zaxira.xlsx
+++ b/Minimal_zaxiralar/Min_Zaxira.xlsx
@@ -8093,10 +8093,10 @@
       </c>
       <c r="E146" s="5" t="n">
         <f aca="false">IF((F146+G146)&gt;0,ROUND((F146+G146)/30,2),"")</f>
-        <v>10</v>
+        <v>16.67</v>
       </c>
       <c r="F146" s="5" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G146" s="5"/>
     </row>
@@ -8115,10 +8115,10 @@
       </c>
       <c r="E147" s="5" t="n">
         <f aca="false">IF((F147+G147)&gt;0,ROUND((F147+G147)/30,2),"")</f>
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="F147" s="5" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="G147" s="5"/>
     </row>
@@ -18534,12 +18534,12 @@
       <c r="D621" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E621" s="5" t="n">
+      <c r="E621" s="5" t="str">
         <f aca="false">IF((F621+G621)&gt;0,ROUND((F621+G621)/30,2),"")</f>
-        <v>13.33</v>
+        <v/>
       </c>
       <c r="F621" s="5" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="G621" s="5"/>
     </row>
@@ -19506,10 +19506,10 @@
       </c>
       <c r="E665" s="5" t="n">
         <f aca="false">IF((F665+G665)&gt;0,ROUND((F665+G665)/30,2),"")</f>
-        <v>13.33</v>
+        <v>6.67</v>
       </c>
       <c r="F665" s="5" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="G665" s="5"/>
     </row>
@@ -19856,12 +19856,12 @@
       <c r="D681" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E681" s="5" t="n">
+      <c r="E681" s="5" t="str">
         <f aca="false">IF((F681+G681)&gt;0,ROUND((F681+G681)/30,2),"")</f>
-        <v>1.67</v>
+        <v/>
       </c>
       <c r="F681" s="5" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G681" s="5"/>
     </row>
@@ -20186,12 +20186,12 @@
       <c r="D696" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E696" s="5" t="n">
+      <c r="E696" s="5" t="str">
         <f aca="false">IF((F696+G696)&gt;0,ROUND((F696+G696)/30,2),"")</f>
-        <v>3.33</v>
+        <v/>
       </c>
       <c r="F696" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G696" s="5"/>
     </row>

</xml_diff>

<commit_message>
Buyurtma excelga Min Zaxira ustuni va jonli formula qoshildi
</commit_message>
<xml_diff>
--- a/Minimal_zaxiralar/Min_Zaxira.xlsx
+++ b/Minimal_zaxiralar/Min_Zaxira.xlsx
@@ -23312,10 +23312,10 @@
       </c>
       <c r="E838" s="5" t="n">
         <f aca="false">IF((F838+G838)&gt;0,ROUND((F838+G838)/30,2),"")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F838" s="5" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="G838" s="5"/>
     </row>
@@ -23638,14 +23638,14 @@
         <v>75</v>
       </c>
       <c r="D853" s="8" t="s">
-        <v>224</v>
+        <v>12</v>
       </c>
       <c r="E853" s="5" t="n">
         <f aca="false">IF((F853+G853)&gt;0,ROUND((F853+G853)/30,2),"")</f>
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="F853" s="5" t="n">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="G853" s="5"/>
     </row>
@@ -23730,10 +23730,10 @@
       </c>
       <c r="E857" s="5" t="n">
         <f aca="false">IF((F857+G857)&gt;0,ROUND((F857+G857)/30,2),"")</f>
-        <v>3.33</v>
+        <v>1.67</v>
       </c>
       <c r="F857" s="5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G857" s="5"/>
     </row>
@@ -23838,10 +23838,7 @@
       <c r="D862" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E862" s="5" t="str">
-        <f aca="false">IF((F862+G862)&gt;0,ROUND((F862+G862)/30,2),"")</f>
-        <v/>
-      </c>
+      <c r="E862" s="5"/>
       <c r="F862" s="5" t="n">
         <v>0</v>
       </c>
@@ -24012,14 +24009,14 @@
         <v>75</v>
       </c>
       <c r="D870" s="8" t="s">
-        <v>224</v>
+        <v>12</v>
       </c>
       <c r="E870" s="5" t="n">
         <f aca="false">IF((F870+G870)&gt;0,ROUND((F870+G870)/30,2),"")</f>
-        <v>6.67</v>
+        <v>3.33</v>
       </c>
       <c r="F870" s="5" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="G870" s="5"/>
     </row>
@@ -24500,10 +24497,10 @@
       </c>
       <c r="E892" s="5" t="n">
         <f aca="false">IF((F892+G892)&gt;0,ROUND((F892+G892)/30,2),"")</f>
-        <v>3.33</v>
+        <v>1.67</v>
       </c>
       <c r="F892" s="5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G892" s="5"/>
     </row>
@@ -24566,10 +24563,10 @@
       </c>
       <c r="E895" s="5" t="n">
         <f aca="false">IF((F895+G895)&gt;0,ROUND((F895+G895)/30,2),"")</f>
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="F895" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G895" s="5"/>
     </row>
@@ -34511,10 +34508,10 @@
       <c r="D1384" s="9"/>
       <c r="E1384" s="5" t="n">
         <f aca="false">IF((F1384+G1384)&gt;0,ROUND((F1384+G1384)/30,2),"")</f>
-        <v>1.67</v>
+        <v>1.33</v>
       </c>
       <c r="F1384" s="5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G1384" s="5"/>
     </row>
@@ -34531,10 +34528,10 @@
       <c r="D1385" s="9"/>
       <c r="E1385" s="5" t="n">
         <f aca="false">IF((F1385+G1385)&gt;0,ROUND((F1385+G1385)/30,2),"")</f>
-        <v>1.67</v>
+        <v>1</v>
       </c>
       <c r="F1385" s="5" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G1385" s="5"/>
     </row>
@@ -34791,12 +34788,12 @@
         <v>75</v>
       </c>
       <c r="D1398" s="9"/>
-      <c r="E1398" s="5" t="n">
+      <c r="E1398" s="5" t="str">
         <f aca="false">IF((F1398+G1398)&gt;0,ROUND((F1398+G1398)/30,2),"")</f>
-        <v>1</v>
+        <v/>
       </c>
       <c r="F1398" s="5" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G1398" s="5"/>
     </row>

</xml_diff>